<commit_message>
Made columns more readable
</commit_message>
<xml_diff>
--- a/data/results/regression_h3_output.xlsx
+++ b/data/results/regression_h3_output.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/33119cfcffe101ac/Documents/Thesis/Thesis folder/conversational-group-rec-eval/data/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="82" documentId="11_77C4DED7983AE929E6F075CAC3C9CFF80A486F74" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C3D7BC92-9051-4354-8AC7-267113FC86F1}"/>
+  <xr:revisionPtr revIDLastSave="85" documentId="11_77C4DED7983AE929E6F075CAC3C9CFF80A486F74" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E518CC75-111C-4AFD-9E13-B7FA45B303CC}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8280" yWindow="4575" windowWidth="17280" windowHeight="9960" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -267,6 +267,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -555,13 +559,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="47.88671875" customWidth="1"/>
-    <col min="2" max="2" width="14.44140625" customWidth="1"/>
+    <col min="1" max="1" width="47.85546875" customWidth="1"/>
+    <col min="2" max="2" width="14.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -569,7 +573,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -577,7 +581,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -585,7 +589,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -593,7 +597,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -601,7 +605,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -609,7 +613,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -625,18 +629,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="61.109375" customWidth="1"/>
-    <col min="2" max="2" width="14.109375" customWidth="1"/>
-    <col min="3" max="3" width="13.44140625" customWidth="1"/>
-    <col min="4" max="4" width="12.21875" customWidth="1"/>
-    <col min="5" max="5" width="12.44140625" customWidth="1"/>
-    <col min="6" max="6" width="11.5546875" customWidth="1"/>
-    <col min="7" max="7" width="12.77734375" customWidth="1"/>
+    <col min="1" max="1" width="61.140625" customWidth="1"/>
+    <col min="2" max="2" width="14.140625" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" customWidth="1"/>
+    <col min="4" max="4" width="12.28515625" customWidth="1"/>
+    <col min="5" max="5" width="12.42578125" customWidth="1"/>
+    <col min="6" max="6" width="11.5703125" customWidth="1"/>
+    <col min="7" max="7" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
@@ -659,7 +663,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -682,7 +686,7 @@
         <v>-2.3958306535096899E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -705,7 +709,7 @@
         <v>-1.9828488186468572E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -728,7 +732,7 @@
         <v>-4.1123544493333261E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -751,7 +755,7 @@
         <v>0.12706268504692461</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -774,7 +778,7 @@
         <v>1.586736196862143</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -797,7 +801,7 @@
         <v>0.24068580804178341</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>22</v>
       </c>
@@ -820,7 +824,7 @@
         <v>2.4163528491829709E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>23</v>
       </c>
@@ -851,19 +855,19 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="54.5546875" customWidth="1"/>
+    <col min="1" max="1" width="56.7109375" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="14.21875" customWidth="1"/>
-    <col min="4" max="4" width="13.88671875" customWidth="1"/>
-    <col min="5" max="5" width="14.33203125" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" customWidth="1"/>
+    <col min="4" max="4" width="13.85546875" customWidth="1"/>
+    <col min="5" max="5" width="14.28515625" customWidth="1"/>
     <col min="6" max="6" width="15" customWidth="1"/>
-    <col min="7" max="7" width="15.109375" customWidth="1"/>
+    <col min="7" max="7" width="15.140625" customWidth="1"/>
     <col min="8" max="8" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
@@ -889,7 +893,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -912,7 +916,7 @@
         <v>0.1242858444174675</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -935,7 +939,7 @@
         <v>1.2889428137128491E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -958,7 +962,7 @@
         <v>3.492978492326853E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -981,7 +985,7 @@
         <v>0.10939349826722861</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -1004,7 +1008,7 @@
         <v>1.696485844753898</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -1027,7 +1031,7 @@
         <v>0.15563167253206839</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>22</v>
       </c>
@@ -1050,7 +1054,7 @@
         <v>2.17244111181213E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>23</v>
       </c>
@@ -1073,7 +1077,7 @@
         <v>0.52902901683538395</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>25</v>
       </c>
@@ -1099,7 +1103,7 @@
         <v>7.8412761706782389E-93</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>26</v>
       </c>
@@ -1125,7 +1129,7 @@
         <v>0.6711644198228196</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>27</v>
       </c>
@@ -1151,7 +1155,7 @@
         <v>1.049947258083123E-150</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>28</v>
       </c>
@@ -1185,13 +1189,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B19"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.21875" customWidth="1"/>
+    <col min="1" max="1" width="25.28515625" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
@@ -1199,7 +1203,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>31</v>
       </c>
@@ -1207,7 +1211,7 @@
         <v>8510</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>32</v>
       </c>
@@ -1215,7 +1219,7 @@
         <v>1374</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>33</v>
       </c>
@@ -1223,7 +1227,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>34</v>
       </c>
@@ -1231,7 +1235,7 @@
         <v>0.40722698924116918</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>35</v>
       </c>
@@ -1239,7 +1243,7 @@
         <v>0.53001964529196965</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>36</v>
       </c>
@@ -1247,7 +1251,7 @@
         <v>0.1227926560508005</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>37</v>
       </c>
@@ -1255,7 +1259,7 @@
         <v>0.4067389380678792</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>38</v>
       </c>
@@ -1263,7 +1267,7 @@
         <v>0.52941129227928574</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>39</v>
       </c>
@@ -1271,7 +1275,7 @@
         <v>2417.2617899774232</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>40</v>
       </c>
@@ -1279,7 +1283,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>41</v>
       </c>
@@ -1287,7 +1291,7 @@
         <v>1673.7257665341081</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>42</v>
       </c>
@@ -1295,15 +1299,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>43</v>
       </c>
       <c r="B14">
-        <v>591.5891706099892</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+        <v>591.58917060998897</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>44</v>
       </c>
@@ -1311,7 +1315,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>45</v>
       </c>
@@ -1319,7 +1323,7 @@
         <v>1373</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>46</v>
       </c>
@@ -1327,7 +1331,7 @@
         <v>8.4077408497699146E-297</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>47</v>
       </c>
@@ -1335,7 +1339,7 @@
         <v>555.07213262560731</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>48</v>
       </c>
@@ -1351,13 +1355,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:B13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="58.77734375" customWidth="1"/>
-    <col min="2" max="2" width="16.33203125" customWidth="1"/>
+    <col min="1" max="1" width="58.7109375" customWidth="1"/>
+    <col min="2" max="2" width="16.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
@@ -1365,7 +1369,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -1373,7 +1377,7 @@
         <v>259.27703974118151</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -1381,7 +1385,7 @@
         <v>6.3244883794338902</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -1389,7 +1393,7 @@
         <v>6.7685234245393744</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -1397,7 +1401,7 @@
         <v>5.0292323729809887</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -1405,7 +1409,7 @@
         <v>1.1390305392766999</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -1413,7 +1417,7 @@
         <v>1.2111300720869349</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>22</v>
       </c>
@@ -1421,7 +1425,7 @@
         <v>1.217274928206046</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>23</v>
       </c>
@@ -1429,7 +1433,7 @@
         <v>1.275536997633244</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>25</v>
       </c>
@@ -1437,7 +1441,7 @@
         <v>1.51585294317784</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>26</v>
       </c>
@@ -1445,7 +1449,7 @@
         <v>1.3238996114754371</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>27</v>
       </c>
@@ -1453,7 +1457,7 @@
         <v>1.299562973755634</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>28</v>
       </c>
@@ -1469,18 +1473,18 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="60.109375" customWidth="1"/>
-    <col min="2" max="2" width="14.88671875" customWidth="1"/>
-    <col min="3" max="3" width="16.5546875" customWidth="1"/>
-    <col min="4" max="4" width="13.77734375" customWidth="1"/>
-    <col min="5" max="5" width="13.33203125" customWidth="1"/>
-    <col min="6" max="6" width="15.109375" customWidth="1"/>
-    <col min="7" max="7" width="14.33203125" customWidth="1"/>
+    <col min="1" max="1" width="60.140625" customWidth="1"/>
+    <col min="2" max="2" width="14.85546875" customWidth="1"/>
+    <col min="3" max="3" width="16.5703125" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" customWidth="1"/>
+    <col min="5" max="5" width="13.28515625" customWidth="1"/>
+    <col min="6" max="6" width="15.140625" customWidth="1"/>
+    <col min="7" max="7" width="14.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
@@ -1503,7 +1507,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -1526,7 +1530,7 @@
         <v>0.13410707562862079</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -1549,7 +1553,7 @@
         <v>-1.06015863409819E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -1572,7 +1576,7 @@
         <v>-1.382369989193733E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -1595,7 +1599,7 @@
         <v>-1.04009339474763E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -1618,7 +1622,7 @@
         <v>3.0977509647085811E-3</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>22</v>
       </c>
@@ -1641,7 +1645,7 @@
         <v>-2.825190258857042E-5</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -1664,7 +1668,7 @@
         <v>1.7112989739023539E-3</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>26</v>
       </c>
@@ -1687,7 +1691,7 @@
         <v>9.9429571404526049E-4</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>27</v>
       </c>
@@ -1710,7 +1714,7 @@
         <v>1.6423870574353589E-3</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>28</v>
       </c>
@@ -1741,17 +1745,17 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:G17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.21875" customWidth="1"/>
-    <col min="2" max="2" width="17.109375" customWidth="1"/>
-    <col min="3" max="3" width="16.21875" customWidth="1"/>
-    <col min="4" max="4" width="12.88671875" customWidth="1"/>
+    <col min="1" max="1" width="11.28515625" customWidth="1"/>
+    <col min="2" max="2" width="17.140625" customWidth="1"/>
+    <col min="3" max="3" width="16.28515625" customWidth="1"/>
+    <col min="4" max="4" width="12.85546875" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="10.5546875" customWidth="1"/>
+    <col min="6" max="6" width="10.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>50</v>
       </c>
@@ -1774,7 +1778,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>51</v>
       </c>
@@ -1797,7 +1801,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>51</v>
       </c>
@@ -1820,7 +1824,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>51</v>
       </c>
@@ -1843,7 +1847,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>51</v>
       </c>
@@ -1866,7 +1870,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>52</v>
       </c>
@@ -1889,7 +1893,7 @@
         <v>3290</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>52</v>
       </c>
@@ -1912,7 +1916,7 @@
         <v>3290</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>52</v>
       </c>
@@ -1935,7 +1939,7 @@
         <v>3290</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>52</v>
       </c>
@@ -1958,7 +1962,7 @@
         <v>3290</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>53</v>
       </c>
@@ -1981,7 +1985,7 @@
         <v>2982</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>53</v>
       </c>
@@ -2004,7 +2008,7 @@
         <v>2982</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>53</v>
       </c>
@@ -2027,7 +2031,7 @@
         <v>2982</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>53</v>
       </c>
@@ -2050,7 +2054,7 @@
         <v>2982</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>54</v>
       </c>
@@ -2073,7 +2077,7 @@
         <v>1858</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>54</v>
       </c>
@@ -2096,7 +2100,7 @@
         <v>1858</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>54</v>
       </c>
@@ -2119,7 +2123,7 @@
         <v>1858</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>54</v>
       </c>
@@ -2150,18 +2154,18 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:H13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="55.44140625" customWidth="1"/>
-    <col min="2" max="2" width="15.6640625" customWidth="1"/>
-    <col min="3" max="3" width="17.5546875" customWidth="1"/>
-    <col min="4" max="5" width="13.33203125" customWidth="1"/>
-    <col min="6" max="6" width="14.21875" customWidth="1"/>
-    <col min="7" max="7" width="12.44140625" customWidth="1"/>
+    <col min="1" max="1" width="57" customWidth="1"/>
+    <col min="2" max="2" width="15.7109375" customWidth="1"/>
+    <col min="3" max="3" width="17.5703125" customWidth="1"/>
+    <col min="4" max="5" width="13.28515625" customWidth="1"/>
+    <col min="6" max="6" width="14.28515625" customWidth="1"/>
+    <col min="7" max="7" width="12.42578125" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
@@ -2187,7 +2191,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -2210,7 +2214,7 @@
         <v>0.12892169785247121</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -2233,7 +2237,7 @@
         <v>1.6929156535693161E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -2256,7 +2260,7 @@
         <v>4.044648899515467E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -2279,7 +2283,7 @@
         <v>0.10475610753337181</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -2302,7 +2306,7 @@
         <v>1.7232377495489259</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -2325,7 +2329,7 @@
         <v>0.17668933284119209</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>22</v>
       </c>
@@ -2348,7 +2352,7 @@
         <v>2.245758487541143E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>23</v>
       </c>
@@ -2371,7 +2375,7 @@
         <v>0.54626905305062479</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>25</v>
       </c>
@@ -2397,7 +2401,7 @@
         <v>7.2973714040969903E-66</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>26</v>
       </c>
@@ -2423,7 +2427,7 @@
         <v>0.9916546509516424</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>27</v>
       </c>
@@ -2449,7 +2453,7 @@
         <v>2.5606555430614181E-115</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>28</v>
       </c>

</xml_diff>